<commit_message>
Update Golden Set Texas AI Act
</commit_message>
<xml_diff>
--- a/Golden_Set_Texas_AI_Act_552_053.xlsx
+++ b/Golden_Set_Texas_AI_Act_552_053.xlsx
@@ -138,7 +138,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -349,10 +349,10 @@
       <c r="A2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="2" t="s">
         <v>4</v>
       </c>
     </row>
@@ -360,15 +360,11 @@
       <c r="A3" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="0"/>
-      <c r="C3" s="0"/>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="0"/>
-      <c r="C4" s="0"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
Update Golden Set Texas AI Act and remove temporary file
</commit_message>
<xml_diff>
--- a/Golden_Set_Texas_AI_Act_552_053.xlsx
+++ b/Golden_Set_Texas_AI_Act_552_053.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" dateCompatibility="false"/>
+  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
@@ -222,37 +222,37 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="000000"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="18a303"/>
+        <a:srgbClr val="18A303"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="0369a3"/>
+        <a:srgbClr val="0369A3"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="a33e03"/>
+        <a:srgbClr val="A33E03"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8e03a3"/>
+        <a:srgbClr val="8E03A3"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="c99c00"/>
+        <a:srgbClr val="C99C00"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="c9211e"/>
+        <a:srgbClr val="C9211E"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ee"/>
+        <a:srgbClr val="0000EE"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="551a8b"/>
+        <a:srgbClr val="551A8B"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">

</xml_diff>